<commit_message>
Updated NEMO analysis and report
</commit_message>
<xml_diff>
--- a/Results/single_algorithm/NEMO/Supplement/Chisq_tests.xlsx
+++ b/Results/single_algorithm/NEMO/Supplement/Chisq_tests.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="44">
   <si>
     <t xml:space="preserve">Comparison</t>
   </si>
@@ -29,124 +29,121 @@
     <t xml:space="preserve">Vital status vs NEMO cluster</t>
   </si>
   <si>
-    <t xml:space="preserve">0.0325215154636905</t>
-  </si>
-  <si>
-    <t xml:space="preserve">27.897608818537</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.098</t>
+    <t xml:space="preserve">0.890338197652804</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.61184451160197</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0</t>
   </si>
   <si>
     <t xml:space="preserve">Ethnicity vs NEMO cluster</t>
   </si>
   <si>
-    <t xml:space="preserve">0.820900073363862</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10.8126330778714</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0</t>
+    <t xml:space="preserve">0.747007647675884</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.09841355225045</t>
   </si>
   <si>
     <t xml:space="preserve">Race vs NEMO cluster</t>
   </si>
   <si>
-    <t xml:space="preserve">0.000388803590033632</t>
-  </si>
-  <si>
-    <t xml:space="preserve">65.8882463867847</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.117</t>
+    <t xml:space="preserve">8.95703286713928e-05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">58.9553760993816</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.138</t>
   </si>
   <si>
     <t xml:space="preserve">Lymph node status vs NEMO cluster</t>
   </si>
   <si>
-    <t xml:space="preserve">0.34027564940234</t>
-  </si>
-  <si>
-    <t xml:space="preserve">17.724483013335</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.037</t>
+    <t xml:space="preserve">0.291164371242248</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9.64057266311515</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.057</t>
   </si>
   <si>
     <t xml:space="preserve">Histology vs NEMO cluster</t>
   </si>
   <si>
-    <t xml:space="preserve">2.40242490696416e-26</t>
-  </si>
-  <si>
-    <t xml:space="preserve">265.380416407111</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.202</t>
+    <t xml:space="preserve">3.53698424452423e-28</t>
+  </si>
+  <si>
+    <t xml:space="preserve">260.768517836023</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.218</t>
   </si>
   <si>
     <t xml:space="preserve">Menopausal status vs NEMO cluster</t>
   </si>
   <si>
-    <t xml:space="preserve">0.657343854526214</t>
-  </si>
-  <si>
-    <t xml:space="preserve">28.2419342095528</t>
+    <t xml:space="preserve">0.701700575354753</t>
+  </si>
+  <si>
+    <t xml:space="preserve">19.9132152657521</t>
   </si>
   <si>
     <t xml:space="preserve">PR status vs NEMO cluster</t>
   </si>
   <si>
-    <t xml:space="preserve">8.27837837108531e-38</t>
-  </si>
-  <si>
-    <t xml:space="preserve">241.407323148239</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.341</t>
+    <t xml:space="preserve">1.64081594738881e-39</t>
+  </si>
+  <si>
+    <t xml:space="preserve">227.992808361467</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.426</t>
   </si>
   <si>
     <t xml:space="preserve">ER status vs NEMO cluster</t>
   </si>
   <si>
-    <t xml:space="preserve">2.01510047369233e-51</t>
-  </si>
-  <si>
-    <t xml:space="preserve">285.991042292466</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.466</t>
+    <t xml:space="preserve">4.65060435375536e-54</t>
+  </si>
+  <si>
+    <t xml:space="preserve">271.53161932236</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.671</t>
   </si>
   <si>
     <t xml:space="preserve">HER2 status vs NEMO cluster</t>
   </si>
   <si>
-    <t xml:space="preserve">3.26388400732618e-05</t>
-  </si>
-  <si>
-    <t xml:space="preserve">74.2861785563774</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.13</t>
+    <t xml:space="preserve">1.5402580668536e-05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">64.3013793528522</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.163</t>
   </si>
   <si>
     <t xml:space="preserve">Metastasis vs NEMO cluster</t>
   </si>
   <si>
-    <t xml:space="preserve">0.467264527869471</t>
-  </si>
-  <si>
-    <t xml:space="preserve">15.7963187326651</t>
+    <t xml:space="preserve">0.900998775198493</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.4765914291658</t>
   </si>
   <si>
     <t xml:space="preserve">Stage vs NEMO cluster</t>
   </si>
   <si>
-    <t xml:space="preserve">0.734554179968769</t>
-  </si>
-  <si>
-    <t xml:space="preserve">26.6416430458449</t>
+    <t xml:space="preserve">0.659131478881233</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20.6524849490866</t>
   </si>
 </sst>
 </file>
@@ -514,133 +511,133 @@
         <v>10</v>
       </c>
       <c r="D3" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B4" t="s">
         <v>12</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
         <v>13</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>14</v>
-      </c>
-      <c r="D4" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5" t="s">
         <v>16</v>
       </c>
-      <c r="B5" t="s">
+      <c r="C5" t="s">
         <v>17</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
         <v>18</v>
-      </c>
-      <c r="D5" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
+        <v>19</v>
+      </c>
+      <c r="B6" t="s">
         <v>20</v>
       </c>
-      <c r="B6" t="s">
+      <c r="C6" t="s">
         <v>21</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
         <v>22</v>
-      </c>
-      <c r="D6" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
+        <v>23</v>
+      </c>
+      <c r="B7" t="s">
         <v>24</v>
       </c>
-      <c r="B7" t="s">
+      <c r="C7" t="s">
         <v>25</v>
       </c>
-      <c r="C7" t="s">
-        <v>26</v>
-      </c>
       <c r="D7" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
+        <v>26</v>
+      </c>
+      <c r="B8" t="s">
         <v>27</v>
       </c>
-      <c r="B8" t="s">
+      <c r="C8" t="s">
         <v>28</v>
       </c>
-      <c r="C8" t="s">
+      <c r="D8" t="s">
         <v>29</v>
-      </c>
-      <c r="D8" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
+        <v>30</v>
+      </c>
+      <c r="B9" t="s">
         <v>31</v>
       </c>
-      <c r="B9" t="s">
+      <c r="C9" t="s">
         <v>32</v>
       </c>
-      <c r="C9" t="s">
+      <c r="D9" t="s">
         <v>33</v>
-      </c>
-      <c r="D9" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
+        <v>34</v>
+      </c>
+      <c r="B10" t="s">
         <v>35</v>
       </c>
-      <c r="B10" t="s">
+      <c r="C10" t="s">
         <v>36</v>
       </c>
-      <c r="C10" t="s">
+      <c r="D10" t="s">
         <v>37</v>
-      </c>
-      <c r="D10" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
+        <v>38</v>
+      </c>
+      <c r="B11" t="s">
         <v>39</v>
       </c>
-      <c r="B11" t="s">
+      <c r="C11" t="s">
         <v>40</v>
       </c>
-      <c r="C11" t="s">
-        <v>41</v>
-      </c>
       <c r="D11" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
+        <v>41</v>
+      </c>
+      <c r="B12" t="s">
         <v>42</v>
       </c>
-      <c r="B12" t="s">
+      <c r="C12" t="s">
         <v>43</v>
       </c>
-      <c r="C12" t="s">
-        <v>44</v>
-      </c>
       <c r="D12" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>